<commit_message>
Adapting of confid, parameter and parsing files to allow handling of well plate data, also uploading more exemplatory data
</commit_message>
<xml_diff>
--- a/data/260511_Wellplate_Photocatalysis_Overview.xlsx
+++ b/data/260511_Wellplate_Photocatalysis_Overview.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jacob/Documents/Water_Splitting/Projects/pyKES-Well-App/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\to86hug\Desktop\HTE plate\pykes\pyKES-Well-App\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7B98B53-BFC5-A54C-A5DD-190BA5B7E2EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C505999-937D-4AD1-9B6E-BBA8CBA799B5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1280" yWindow="2460" windowWidth="28700" windowHeight="15940" xr2:uid="{F5E592D8-4D62-B24E-B288-68BE35DDDD37}"/>
+    <workbookView xWindow="1275" yWindow="2460" windowWidth="28695" windowHeight="15945" xr2:uid="{F5E592D8-4D62-B24E-B288-68BE35DDDD37}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,23 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="60">
   <si>
     <t>Experiment</t>
   </si>
@@ -62,9 +51,6 @@
     <t>Irradiance B [mW/cm2]</t>
   </si>
   <si>
-    <t>Beam combiner [TRUE/FALSE]</t>
-  </si>
-  <si>
     <t>Measurement phase [liquid/gas]</t>
   </si>
   <si>
@@ -86,9 +72,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>Gas phase volume [mL]</t>
-  </si>
-  <si>
     <t>Liquid phase volume [mL]</t>
   </si>
   <si>
@@ -107,9 +90,6 @@
     <t>liquid</t>
   </si>
   <si>
-    <t>2026-03-26_230819_EA-555-Ch2-Robust-3.txt</t>
-  </si>
-  <si>
     <t>group</t>
   </si>
   <si>
@@ -173,13 +153,58 @@
     <t>Well</t>
   </si>
   <si>
-    <t>AE-772</t>
-  </si>
-  <si>
-    <t>File name temperature</t>
-  </si>
-  <si>
-    <t>A1</t>
+    <t>AE-772-1.txt</t>
+  </si>
+  <si>
+    <t>File name calibration</t>
+  </si>
+  <si>
+    <t>calibration.csv</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>AE-772_C1</t>
+  </si>
+  <si>
+    <t>AE-772_B1</t>
+  </si>
+  <si>
+    <t>B1</t>
+  </si>
+  <si>
+    <t>dark blue</t>
+  </si>
+  <si>
+    <t>green</t>
+  </si>
+  <si>
+    <t>dark green</t>
+  </si>
+  <si>
+    <t>red</t>
+  </si>
+  <si>
+    <t>dark red</t>
+  </si>
+  <si>
+    <t>AE-772_D1</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>AE-788_B1</t>
+  </si>
+  <si>
+    <t>AE-788_C1</t>
+  </si>
+  <si>
+    <t>AE-788_D1</t>
+  </si>
+  <si>
+    <t>AE-788-1.txt</t>
   </si>
 </sst>
 </file>
@@ -232,15 +257,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -254,9 +290,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{84101FB2-5380-364F-BE52-83A6609AE9BE}" name="Table1" displayName="Table1" ref="A1:AG174" totalsRowShown="0">
-  <autoFilter ref="A1:AG174" xr:uid="{84101FB2-5380-364F-BE52-83A6609AE9BE}"/>
-  <tableColumns count="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{84101FB2-5380-364F-BE52-83A6609AE9BE}" name="Table1" displayName="Table1" ref="A1:AE174" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:AE174" xr:uid="{84101FB2-5380-364F-BE52-83A6609AE9BE}"/>
+  <tableColumns count="31">
     <tableColumn id="1" xr3:uid="{0F69D98F-F45C-9544-BF7D-68B0AD17E6A9}" name="Experiment"/>
     <tableColumn id="34" xr3:uid="{09DADDBE-3A26-A440-A579-B1C06EACCFE4}" name="Well"/>
     <tableColumn id="2" xr3:uid="{FD5B5509-0AA0-2A49-9666-7F40611BD5F0}" name="group"/>
@@ -278,13 +314,11 @@
     <tableColumn id="9" xr3:uid="{F518EC00-1998-7042-B7C6-3C87845A4480}" name="Irradiance A [mW/cm2]"/>
     <tableColumn id="10" xr3:uid="{050A824F-7BBB-D140-B7A5-B305F07479DD}" name="Irradiation wavelength B [nm]"/>
     <tableColumn id="11" xr3:uid="{6402CA08-B252-F849-A357-F3E827B74D3B}" name="Irradiance B [mW/cm2]"/>
-    <tableColumn id="12" xr3:uid="{A170F6BD-E3C9-9042-B8C4-DB68390CB9E4}" name="Beam combiner [TRUE/FALSE]"/>
     <tableColumn id="14" xr3:uid="{69BA3B85-05E9-E447-8DC3-8A1FB088E183}" name="Temperature [°C]"/>
     <tableColumn id="15" xr3:uid="{2E4E8861-B318-3E47-80A7-51803FD13CD5}" name="Catalyst concentration [g/L]"/>
-    <tableColumn id="43" xr3:uid="{4A3DE809-237A-2E4E-975D-72CB0A88802B}" name="Gas phase volume [mL]"/>
     <tableColumn id="44" xr3:uid="{2A951B80-0DB9-EC46-BE34-A2430E756E1A}" name="Liquid phase volume [mL]"/>
     <tableColumn id="17" xr3:uid="{353F77CA-EAE1-3940-937B-408AE3F5F5A5}" name="File name O2"/>
-    <tableColumn id="35" xr3:uid="{2E1BA3C2-F15F-AB4C-8CF7-1CECA88F8FE2}" name="File name temperature"/>
+    <tableColumn id="35" xr3:uid="{2E1BA3C2-F15F-AB4C-8CF7-1CECA88F8FE2}" name="File name calibration"/>
     <tableColumn id="20" xr3:uid="{32F74BB6-C1D7-1A4C-85E4-1CD8796D6C03}" name="Pyroscience Irradiation start [s]"/>
     <tableColumn id="21" xr3:uid="{DF6B8CAD-6D48-7D4A-929D-B2E9B8917F1C}" name="Pyroscience Irradiation end [s]"/>
     <tableColumn id="23" xr3:uid="{53CFF021-E072-984D-A864-F539B05F85B3}" name="Active"/>
@@ -612,61 +646,63 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{980764FC-9EB3-EA4F-8BCB-174812DC85CB}">
-  <dimension ref="A1:AG2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <dimension ref="A1:AE7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="21.140625" customWidth="1"/>
-    <col min="3" max="3" width="21" customWidth="1"/>
-    <col min="4" max="4" width="27.28515625" customWidth="1"/>
-    <col min="5" max="5" width="29" customWidth="1"/>
-    <col min="6" max="6" width="19.7109375" customWidth="1"/>
-    <col min="7" max="7" width="17.7109375" customWidth="1"/>
-    <col min="8" max="8" width="18.85546875" customWidth="1"/>
-    <col min="9" max="9" width="30.7109375" customWidth="1"/>
-    <col min="10" max="10" width="40.28515625" customWidth="1"/>
-    <col min="11" max="11" width="33.28515625" customWidth="1"/>
-    <col min="12" max="14" width="27.42578125" customWidth="1"/>
-    <col min="15" max="15" width="45.5703125" customWidth="1"/>
-    <col min="16" max="16" width="25.140625" customWidth="1"/>
-    <col min="17" max="17" width="20.28515625" customWidth="1"/>
-    <col min="18" max="18" width="28.28515625" customWidth="1"/>
-    <col min="19" max="19" width="24.7109375" customWidth="1"/>
-    <col min="20" max="20" width="28.5703125" customWidth="1"/>
-    <col min="21" max="21" width="22" customWidth="1"/>
-    <col min="22" max="22" width="28.85546875" customWidth="1"/>
-    <col min="23" max="23" width="17.140625" customWidth="1"/>
-    <col min="24" max="24" width="26.42578125" customWidth="1"/>
-    <col min="25" max="25" width="23.7109375" customWidth="1"/>
-    <col min="26" max="26" width="24.28515625" customWidth="1"/>
-    <col min="27" max="28" width="33.28515625" customWidth="1"/>
-    <col min="29" max="29" width="33" customWidth="1"/>
-    <col min="30" max="30" width="30.28515625" customWidth="1"/>
-    <col min="31" max="31" width="10.28515625" customWidth="1"/>
-    <col min="32" max="32" width="10.7109375" customWidth="1"/>
-    <col min="33" max="33" width="124.140625" customWidth="1"/>
+    <col min="1" max="1" width="13.21875" customWidth="1"/>
+    <col min="2" max="2" width="8.5546875" customWidth="1"/>
+    <col min="3" max="3" width="12.5546875" customWidth="1"/>
+    <col min="4" max="4" width="15.21875" customWidth="1"/>
+    <col min="5" max="5" width="14.77734375" customWidth="1"/>
+    <col min="6" max="6" width="10.33203125" customWidth="1"/>
+    <col min="7" max="7" width="8.77734375" customWidth="1"/>
+    <col min="8" max="8" width="8.88671875" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="10" max="10" width="20.21875" customWidth="1"/>
+    <col min="11" max="11" width="15.21875" customWidth="1"/>
+    <col min="12" max="12" width="13" customWidth="1"/>
+    <col min="13" max="13" width="10" customWidth="1"/>
+    <col min="14" max="14" width="10.6640625" customWidth="1"/>
+    <col min="15" max="15" width="18.5546875" customWidth="1"/>
+    <col min="16" max="16" width="11.33203125" customWidth="1"/>
+    <col min="17" max="17" width="8" customWidth="1"/>
+    <col min="18" max="18" width="14.5546875" customWidth="1"/>
+    <col min="19" max="19" width="9.44140625" customWidth="1"/>
+    <col min="20" max="20" width="9.77734375" customWidth="1"/>
+    <col min="21" max="21" width="5.6640625" customWidth="1"/>
+    <col min="22" max="22" width="6.33203125" customWidth="1"/>
+    <col min="23" max="23" width="9.77734375" customWidth="1"/>
+    <col min="24" max="24" width="8.21875" customWidth="1"/>
+    <col min="25" max="25" width="15.77734375" customWidth="1"/>
+    <col min="26" max="26" width="21.6640625" customWidth="1"/>
+    <col min="27" max="27" width="14.6640625" customWidth="1"/>
+    <col min="28" max="28" width="8.6640625" customWidth="1"/>
+    <col min="29" max="29" width="10.33203125" customWidth="1"/>
+    <col min="30" max="30" width="10.6640625" customWidth="1"/>
+    <col min="31" max="31" width="124.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33">
+    <row r="1" spans="1:31" s="2" customFormat="1" ht="78.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>2</v>
@@ -675,28 +711,28 @@
         <v>3</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="K1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="P1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="N1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="R1" s="1" t="s">
         <v>4</v>
@@ -710,64 +746,58 @@
       <c r="U1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="V1" t="s">
-        <v>8</v>
-      </c>
-      <c r="W1" t="s">
+      <c r="V1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="W1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="Y1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AA1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="AB1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:31">
+      <c r="A2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" t="s">
         <v>16</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="D2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" t="s">
         <v>17</v>
       </c>
-      <c r="AA1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="AC1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="AD1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="AE1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:33">
-      <c r="A2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E2" t="s">
-        <v>19</v>
-      </c>
       <c r="F2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G2" t="s">
         <v>40</v>
-      </c>
-      <c r="G2" t="s">
-        <v>43</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -776,25 +806,25 @@
         <v>1000</v>
       </c>
       <c r="J2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="K2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="L2">
         <v>0.1</v>
       </c>
       <c r="M2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="N2">
         <v>0</v>
       </c>
       <c r="O2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="P2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="Q2">
         <v>1.5</v>
@@ -811,38 +841,510 @@
       <c r="U2">
         <v>170</v>
       </c>
-      <c r="V2" t="b">
+      <c r="V2">
+        <v>20</v>
+      </c>
+      <c r="W2">
         <v>1</v>
       </c>
-      <c r="W2">
+      <c r="X2">
+        <v>2</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA2">
+        <v>900</v>
+      </c>
+      <c r="AB2">
+        <v>8100</v>
+      </c>
+      <c r="AC2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>24</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:31">
+      <c r="A3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
         <v>20</v>
       </c>
-      <c r="X2">
+      <c r="E3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>1000</v>
+      </c>
+      <c r="J3" t="s">
+        <v>19</v>
+      </c>
+      <c r="K3" t="s">
+        <v>29</v>
+      </c>
+      <c r="L3">
+        <v>0.1</v>
+      </c>
+      <c r="M3" t="s">
+        <v>32</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3" t="s">
+        <v>26</v>
+      </c>
+      <c r="P3" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q3">
+        <v>1.5</v>
+      </c>
+      <c r="R3">
+        <v>525</v>
+      </c>
+      <c r="S3">
+        <v>12</v>
+      </c>
+      <c r="T3">
+        <v>625</v>
+      </c>
+      <c r="U3">
+        <v>170</v>
+      </c>
+      <c r="V3">
+        <v>20</v>
+      </c>
+      <c r="W3">
         <v>1</v>
       </c>
-      <c r="Y2">
-        <v>5</v>
-      </c>
-      <c r="Z2">
+      <c r="X3">
         <v>2</v>
       </c>
-      <c r="AA2" t="s">
-        <v>23</v>
-      </c>
-      <c r="AC2">
+      <c r="Y3" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA3">
         <v>900</v>
       </c>
-      <c r="AD2">
+      <c r="AB3">
         <v>8100</v>
       </c>
-      <c r="AE2" t="b">
+      <c r="AC3" t="b">
         <v>1</v>
       </c>
-      <c r="AF2" t="s">
-        <v>27</v>
-      </c>
-      <c r="AG2" t="s">
-        <v>38</v>
+      <c r="AD3" t="s">
+        <v>49</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:31">
+      <c r="A4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>1000</v>
+      </c>
+      <c r="J4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K4" t="s">
+        <v>29</v>
+      </c>
+      <c r="L4">
+        <v>0.1</v>
+      </c>
+      <c r="M4" t="s">
+        <v>32</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4" t="s">
+        <v>26</v>
+      </c>
+      <c r="P4" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q4">
+        <v>1.5</v>
+      </c>
+      <c r="R4">
+        <v>525</v>
+      </c>
+      <c r="S4">
+        <v>12</v>
+      </c>
+      <c r="T4">
+        <v>625</v>
+      </c>
+      <c r="U4">
+        <v>170</v>
+      </c>
+      <c r="V4">
+        <v>20</v>
+      </c>
+      <c r="W4">
+        <v>1</v>
+      </c>
+      <c r="X4">
+        <v>2</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA4">
+        <v>900</v>
+      </c>
+      <c r="AB4">
+        <v>8100</v>
+      </c>
+      <c r="AC4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>50</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:31">
+      <c r="A5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" t="s">
+        <v>40</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>1000</v>
+      </c>
+      <c r="J5" t="s">
+        <v>19</v>
+      </c>
+      <c r="K5" t="s">
+        <v>29</v>
+      </c>
+      <c r="L5">
+        <v>0.1</v>
+      </c>
+      <c r="M5" t="s">
+        <v>32</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5" t="s">
+        <v>26</v>
+      </c>
+      <c r="P5" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q5">
+        <v>1.5</v>
+      </c>
+      <c r="R5">
+        <v>525</v>
+      </c>
+      <c r="S5">
+        <v>12</v>
+      </c>
+      <c r="T5">
+        <v>625</v>
+      </c>
+      <c r="U5">
+        <v>170</v>
+      </c>
+      <c r="V5">
+        <v>20</v>
+      </c>
+      <c r="W5">
+        <v>1</v>
+      </c>
+      <c r="X5">
+        <v>2</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>59</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA5">
+        <v>900</v>
+      </c>
+      <c r="AB5">
+        <v>8100</v>
+      </c>
+      <c r="AC5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD5" t="s">
+        <v>51</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:31">
+      <c r="A6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G6" t="s">
+        <v>40</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>1000</v>
+      </c>
+      <c r="J6" t="s">
+        <v>19</v>
+      </c>
+      <c r="K6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L6">
+        <v>0.1</v>
+      </c>
+      <c r="M6" t="s">
+        <v>32</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P6" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q6">
+        <v>1.5</v>
+      </c>
+      <c r="R6">
+        <v>525</v>
+      </c>
+      <c r="S6">
+        <v>12</v>
+      </c>
+      <c r="T6">
+        <v>625</v>
+      </c>
+      <c r="U6">
+        <v>170</v>
+      </c>
+      <c r="V6">
+        <v>20</v>
+      </c>
+      <c r="W6">
+        <v>1</v>
+      </c>
+      <c r="X6">
+        <v>2</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>59</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA6">
+        <v>900</v>
+      </c>
+      <c r="AB6">
+        <v>8100</v>
+      </c>
+      <c r="AC6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>52</v>
+      </c>
+      <c r="AE6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:31">
+      <c r="A7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G7" t="s">
+        <v>40</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>1000</v>
+      </c>
+      <c r="J7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K7" t="s">
+        <v>29</v>
+      </c>
+      <c r="L7">
+        <v>0.1</v>
+      </c>
+      <c r="M7" t="s">
+        <v>32</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7" t="s">
+        <v>26</v>
+      </c>
+      <c r="P7" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q7">
+        <v>1.5</v>
+      </c>
+      <c r="R7">
+        <v>525</v>
+      </c>
+      <c r="S7">
+        <v>12</v>
+      </c>
+      <c r="T7">
+        <v>625</v>
+      </c>
+      <c r="U7">
+        <v>170</v>
+      </c>
+      <c r="V7">
+        <v>20</v>
+      </c>
+      <c r="W7">
+        <v>1</v>
+      </c>
+      <c r="X7">
+        <v>2</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>59</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA7">
+        <v>900</v>
+      </c>
+      <c r="AB7">
+        <v>8100</v>
+      </c>
+      <c r="AC7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE7" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>